<commit_message>
Implementacion cuerpo y envio de correo
</commit_message>
<xml_diff>
--- a/Reports/Reporte_USD.xlsx
+++ b/Reports/Reporte_USD.xlsx
@@ -533,10 +533,10 @@
         <v>0</v>
       </c>
       <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
         <v>1971.39</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0</v>
       </c>
       <c r="N2" t="n">
         <v>1</v>
@@ -626,10 +626,10 @@
         <v>5228.91</v>
       </c>
       <c r="G4" t="n">
-        <v>5228.91</v>
+        <v>2634.86</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>2594.05</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -680,10 +680,10 @@
         <v>150055.16</v>
       </c>
       <c r="G5" t="n">
-        <v>150039.63</v>
+        <v>146699.17</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>3340.46</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -734,10 +734,10 @@
         <v>3123.39</v>
       </c>
       <c r="G6" t="n">
-        <v>3123.39</v>
+        <v>2675.69</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>447.7</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -1220,10 +1220,10 @@
         <v>6358.8</v>
       </c>
       <c r="G15" t="n">
-        <v>6358.8</v>
+        <v>5900.8</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>458</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
@@ -1334,10 +1334,10 @@
         <v>0</v>
       </c>
       <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="n">
         <v>1990</v>
-      </c>
-      <c r="J17" t="n">
-        <v>0</v>
       </c>
       <c r="K17" t="n">
         <v>0</v>

</xml_diff>